<commit_message>
docs: update syllabus to clarify sustainability connection and classroom culture
</commit_message>
<xml_diff>
--- a/comp364-schedule-8-11-2026.xlsx
+++ b/comp364-schedule-8-11-2026.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BA681B0-13C5-4BA8-B9AE-1B4710C7AA8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -658,53 +658,53 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1014,19 +1014,19 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H37"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="6.140625" style="8" customWidth="1"/>
-    <col min="2" max="2" width="5.140625" style="18" customWidth="1"/>
-    <col min="3" max="3" width="6.42578125" style="13" customWidth="1"/>
-    <col min="4" max="4" width="21.28515625" style="7" customWidth="1"/>
-    <col min="5" max="5" width="7.5703125" style="8" customWidth="1"/>
-    <col min="6" max="6" width="11.7109375" style="8" customWidth="1"/>
-    <col min="7" max="7" width="34.7109375" style="45" customWidth="1"/>
-    <col min="8" max="8" width="37.85546875" customWidth="1"/>
+    <col min="1" max="1" width="6.1796875" style="8" customWidth="1"/>
+    <col min="2" max="2" width="5.1796875" style="18" customWidth="1"/>
+    <col min="3" max="3" width="6.453125" style="13" customWidth="1"/>
+    <col min="4" max="4" width="21.26953125" style="7" customWidth="1"/>
+    <col min="5" max="5" width="7.54296875" style="8" customWidth="1"/>
+    <col min="6" max="6" width="11.7265625" style="8" customWidth="1"/>
+    <col min="7" max="7" width="34.7265625" style="40" customWidth="1"/>
+    <col min="8" max="8" width="37.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="6" customFormat="1" ht="24" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>33</v>
       </c>
@@ -1045,12 +1045,12 @@
       <c r="F1" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="G1" s="39" t="s">
+      <c r="G1" s="34" t="s">
         <v>43</v>
       </c>
       <c r="H1"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="10">
         <v>1</v>
       </c>
@@ -1060,18 +1060,18 @@
       <c r="C2" s="14">
         <v>46266</v>
       </c>
-      <c r="D2" s="34" t="s">
+      <c r="D2" s="49" t="s">
         <v>49</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>5</v>
       </c>
       <c r="F2" s="10"/>
-      <c r="G2" s="40" t="s">
+      <c r="G2" s="35" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="10"/>
       <c r="B3" s="16" t="s">
         <v>36</v>
@@ -1080,16 +1080,16 @@
         <f>C2+3</f>
         <v>46269</v>
       </c>
-      <c r="D3" s="34"/>
+      <c r="D3" s="49"/>
       <c r="E3" s="5" t="s">
         <v>6</v>
       </c>
       <c r="F3" s="10"/>
-      <c r="G3" s="40" t="s">
+      <c r="G3" s="35" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="10">
         <f>A2+1</f>
         <v>2</v>
@@ -1102,16 +1102,16 @@
         <f>C2+7</f>
         <v>46273</v>
       </c>
-      <c r="D4" s="34"/>
+      <c r="D4" s="49"/>
       <c r="E4" s="5" t="s">
         <v>7</v>
       </c>
       <c r="F4" s="10"/>
-      <c r="G4" s="40" t="s">
+      <c r="G4" s="35" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="10"/>
       <c r="B5" s="16" t="str">
         <f>B3</f>
@@ -1121,7 +1121,7 @@
         <f>C3+7</f>
         <v>46276</v>
       </c>
-      <c r="D5" s="34" t="s">
+      <c r="D5" s="49" t="s">
         <v>47</v>
       </c>
       <c r="E5" s="5" t="s">
@@ -1130,11 +1130,11 @@
       <c r="F5" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="G5" s="40" t="s">
+      <c r="G5" s="35" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="10">
         <f t="shared" ref="A6" si="0">A4+1</f>
         <v>3</v>
@@ -1147,16 +1147,16 @@
         <f t="shared" ref="C6:C33" si="2">C4+7</f>
         <v>46280</v>
       </c>
-      <c r="D6" s="34"/>
+      <c r="D6" s="49"/>
       <c r="E6" s="5" t="s">
         <v>9</v>
       </c>
       <c r="F6" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="G6" s="41"/>
-    </row>
-    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="G6" s="36"/>
+    </row>
+    <row r="7" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="10"/>
       <c r="B7" s="16" t="str">
         <f t="shared" si="1"/>
@@ -1173,11 +1173,11 @@
         <v>10</v>
       </c>
       <c r="F7" s="10"/>
-      <c r="G7" s="40" t="s">
+      <c r="G7" s="35" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="10">
         <f t="shared" ref="A8" si="3">A6+1</f>
         <v>4</v>
@@ -1190,7 +1190,7 @@
         <f t="shared" si="2"/>
         <v>46287</v>
       </c>
-      <c r="D8" s="34" t="s">
+      <c r="D8" s="49" t="s">
         <v>48</v>
       </c>
       <c r="E8" s="5" t="s">
@@ -1199,9 +1199,9 @@
       <c r="F8" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="G8" s="42"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G8" s="37"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="10"/>
       <c r="B9" s="16" t="str">
         <f t="shared" si="1"/>
@@ -1211,18 +1211,18 @@
         <f t="shared" si="2"/>
         <v>46290</v>
       </c>
-      <c r="D9" s="34"/>
+      <c r="D9" s="49"/>
       <c r="E9" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F9" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="G9" s="40" t="s">
+      <c r="G9" s="35" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="33" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="10"/>
       <c r="B10" s="16" t="s">
         <v>72</v>
@@ -1230,16 +1230,16 @@
       <c r="C10" s="14">
         <v>46291</v>
       </c>
-      <c r="D10" s="35" t="s">
+      <c r="D10" s="42" t="s">
         <v>62</v>
       </c>
-      <c r="E10" s="38" t="s">
+      <c r="E10" s="41" t="s">
         <v>73</v>
       </c>
-      <c r="F10" s="38"/>
-      <c r="G10" s="38"/>
-    </row>
-    <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F10" s="41"/>
+      <c r="G10" s="41"/>
+    </row>
+    <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="10">
         <f t="shared" ref="A11" si="4">A8+1</f>
         <v>5</v>
@@ -1252,16 +1252,16 @@
         <f>C8+7</f>
         <v>46294</v>
       </c>
-      <c r="D11" s="36"/>
+      <c r="D11" s="43"/>
       <c r="E11" s="5" t="s">
         <v>13</v>
       </c>
       <c r="F11" s="10"/>
-      <c r="G11" s="42" t="s">
+      <c r="G11" s="37" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="10"/>
       <c r="B12" s="16" t="str">
         <f>B9</f>
@@ -1271,18 +1271,18 @@
         <f>C9+7</f>
         <v>46297</v>
       </c>
-      <c r="D12" s="36"/>
+      <c r="D12" s="43"/>
       <c r="E12" s="5" t="s">
         <v>14</v>
       </c>
       <c r="F12" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="G12" s="40" t="s">
+      <c r="G12" s="35" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="38.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="10">
         <f t="shared" ref="A13" si="5">A11+1</f>
         <v>6</v>
@@ -1295,16 +1295,16 @@
         <f t="shared" si="2"/>
         <v>46301</v>
       </c>
-      <c r="D13" s="37"/>
+      <c r="D13" s="44"/>
       <c r="E13" s="5" t="s">
         <v>15</v>
       </c>
       <c r="F13" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="G13" s="40"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G13" s="35"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="10"/>
       <c r="B14" s="16" t="str">
         <f t="shared" si="1"/>
@@ -1323,9 +1323,9 @@
       <c r="F14" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="G14" s="40"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G14" s="35"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="10">
         <f t="shared" ref="A15" si="6">A13+1</f>
         <v>7</v>
@@ -1345,9 +1345,9 @@
         <v>17</v>
       </c>
       <c r="F15" s="10"/>
-      <c r="G15" s="41"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G15" s="36"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="10"/>
       <c r="B16" s="16" t="str">
         <f t="shared" si="1"/>
@@ -1364,11 +1364,11 @@
         <v>18</v>
       </c>
       <c r="F16" s="10"/>
-      <c r="G16" s="40" t="s">
+      <c r="G16" s="35" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="10"/>
       <c r="B17" s="16" t="str">
         <f t="shared" si="1"/>
@@ -1383,9 +1383,9 @@
       </c>
       <c r="E17" s="9"/>
       <c r="F17" s="21"/>
-      <c r="G17" s="40"/>
-    </row>
-    <row r="18" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G17" s="35"/>
+    </row>
+    <row r="18" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="10">
         <v>8</v>
       </c>
@@ -1397,46 +1397,46 @@
         <f t="shared" si="2"/>
         <v>46318</v>
       </c>
-      <c r="D18" s="34" t="s">
+      <c r="D18" s="49" t="s">
         <v>41</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>19</v>
       </c>
       <c r="F18" s="10"/>
-      <c r="G18" s="41"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G18" s="36"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="10"/>
-      <c r="B19" s="46" t="str">
+      <c r="B19" s="45" t="str">
         <f>B17</f>
         <v>Tue</v>
       </c>
-      <c r="C19" s="48">
+      <c r="C19" s="47">
         <f>C17+7</f>
         <v>46322</v>
       </c>
-      <c r="D19" s="34"/>
+      <c r="D19" s="49"/>
       <c r="E19" s="5" t="s">
         <v>20</v>
       </c>
       <c r="F19" s="10"/>
-      <c r="G19" s="40" t="s">
+      <c r="G19" s="35" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="10"/>
-      <c r="B20" s="47"/>
-      <c r="C20" s="49"/>
-      <c r="D20" s="34"/>
-      <c r="E20" s="38" t="s">
+      <c r="B20" s="46"/>
+      <c r="C20" s="48"/>
+      <c r="D20" s="49"/>
+      <c r="E20" s="41" t="s">
         <v>91</v>
       </c>
-      <c r="F20" s="38"/>
-      <c r="G20" s="38"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F20" s="41"/>
+      <c r="G20" s="41"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="10">
         <f>A18+1</f>
         <v>9</v>
@@ -1449,16 +1449,16 @@
         <f>C18+7</f>
         <v>46325</v>
       </c>
-      <c r="D21" s="34"/>
+      <c r="D21" s="49"/>
       <c r="E21" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F21" s="10"/>
-      <c r="G21" s="40" t="s">
+      <c r="G21" s="35" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="10"/>
       <c r="B22" s="16" t="str">
         <f>B19</f>
@@ -1475,11 +1475,11 @@
         <v>22</v>
       </c>
       <c r="F22" s="26"/>
-      <c r="G22" s="40" t="s">
+      <c r="G22" s="35" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" s="10">
         <f t="shared" ref="A23" si="7">A21+1</f>
         <v>10</v>
@@ -1501,9 +1501,9 @@
       <c r="F23" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="G23" s="40"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G23" s="35"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="10"/>
       <c r="B24" s="16" t="str">
         <f t="shared" si="1"/>
@@ -1513,7 +1513,7 @@
         <f t="shared" si="2"/>
         <v>46336</v>
       </c>
-      <c r="D24" s="34" t="s">
+      <c r="D24" s="49" t="s">
         <v>66</v>
       </c>
       <c r="E24" s="5" t="s">
@@ -1522,9 +1522,9 @@
       <c r="F24" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="G24" s="41"/>
-    </row>
-    <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G24" s="36"/>
+    </row>
+    <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="10">
         <f t="shared" ref="A25" si="8">A23+1</f>
         <v>11</v>
@@ -1537,16 +1537,16 @@
         <f t="shared" si="2"/>
         <v>46339</v>
       </c>
-      <c r="D25" s="34"/>
+      <c r="D25" s="49"/>
       <c r="E25" s="5" t="s">
         <v>25</v>
       </c>
       <c r="F25" s="10"/>
-      <c r="G25" s="40" t="s">
+      <c r="G25" s="35" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="10"/>
       <c r="B26" s="16" t="str">
         <f t="shared" si="1"/>
@@ -1563,11 +1563,11 @@
         <v>26</v>
       </c>
       <c r="F26" s="22"/>
-      <c r="G26" s="40" t="s">
+      <c r="G26" s="35" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="10">
         <f t="shared" ref="A27" si="9">A25+1</f>
         <v>12</v>
@@ -1589,9 +1589,9 @@
       <c r="F27" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="G27" s="41"/>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G27" s="36"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="10"/>
       <c r="B28" s="16" t="str">
         <f t="shared" si="1"/>
@@ -1610,11 +1610,11 @@
       <c r="F28" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="G28" s="40" t="s">
+      <c r="G28" s="35" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" s="10"/>
       <c r="B29" s="16" t="str">
         <f t="shared" si="1"/>
@@ -1629,9 +1629,9 @@
       </c>
       <c r="E29" s="9"/>
       <c r="F29" s="10"/>
-      <c r="G29" s="40"/>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G29" s="35"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="10">
         <f>A27+1</f>
         <v>13</v>
@@ -1651,9 +1651,9 @@
         <v>29</v>
       </c>
       <c r="F30" s="10"/>
-      <c r="G30" s="43"/>
-    </row>
-    <row r="31" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G30" s="38"/>
+    </row>
+    <row r="31" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A31" s="19"/>
       <c r="B31" s="17" t="str">
         <f t="shared" si="1"/>
@@ -1672,12 +1672,12 @@
       <c r="F31" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="G31" s="40" t="s">
+      <c r="G31" s="35" t="s">
         <v>88</v>
       </c>
       <c r="H31"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="10">
         <f t="shared" ref="A32" si="10">A30+1</f>
         <v>14</v>
@@ -1697,11 +1697,11 @@
         <v>31</v>
       </c>
       <c r="F32" s="19"/>
-      <c r="G32" s="40" t="s">
+      <c r="G32" s="35" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="10"/>
       <c r="B33" s="16" t="str">
         <f t="shared" si="1"/>
@@ -1720,9 +1720,9 @@
       <c r="F33" s="33" t="s">
         <v>70</v>
       </c>
-      <c r="G33" s="41"/>
-    </row>
-    <row r="34" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="G33" s="36"/>
+    </row>
+    <row r="34" spans="1:7" ht="39" x14ac:dyDescent="0.35">
       <c r="A34" s="10"/>
       <c r="B34" s="16" t="s">
         <v>36</v>
@@ -1737,27 +1737,27 @@
       <c r="F34" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="G34" s="40"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G34" s="35"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="F35" s="6"/>
-      <c r="G35" s="44"/>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G35" s="39"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="D37"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="D2:D4"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="D18:D21"/>
     <mergeCell ref="E10:G10"/>
     <mergeCell ref="D10:D13"/>
     <mergeCell ref="E20:G20"/>
     <mergeCell ref="B19:B20"/>
     <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D2:D4"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="D18:D21"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>